<commit_message>
Add file from private repo
</commit_message>
<xml_diff>
--- a/CryCompanywiseStockReport_1.xlsx
+++ b/CryCompanywiseStockReport_1.xlsx
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="M1" t="n">
-        <v>46075</v>
+        <v>46076</v>
       </c>
     </row>
     <row r="2">
@@ -15156,7 +15156,7 @@
         <v>408</v>
       </c>
       <c r="B512" t="n">
-        <v>60022</v>
+        <v>64830</v>
       </c>
       <c r="C512" t="inlineStr">
         <is>
@@ -15167,13 +15167,13 @@
         <v>32.83</v>
       </c>
       <c r="E512" t="n">
-        <v>37.22</v>
+        <v>34.9</v>
       </c>
       <c r="F512" t="n">
-        <v>-113</v>
+        <v>83</v>
       </c>
       <c r="G512" t="n">
-        <v>-3709.79</v>
+        <v>2724.89</v>
       </c>
       <c r="H512" t="inlineStr"/>
       <c r="I512" t="inlineStr"/>
@@ -15187,7 +15187,7 @@
         <v>409</v>
       </c>
       <c r="B513" t="n">
-        <v>64830</v>
+        <v>60022</v>
       </c>
       <c r="C513" t="inlineStr">
         <is>
@@ -15198,13 +15198,13 @@
         <v>32.83</v>
       </c>
       <c r="E513" t="n">
-        <v>34.9</v>
+        <v>37.22</v>
       </c>
       <c r="F513" t="n">
-        <v>83</v>
+        <v>-113</v>
       </c>
       <c r="G513" t="n">
-        <v>2724.89</v>
+        <v>-3709.79</v>
       </c>
       <c r="H513" t="inlineStr"/>
       <c r="I513" t="inlineStr"/>

</xml_diff>